<commit_message>
Research: add EU shops without Croatian site that ship to Croatia
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LFT8mCLN1P2JpRsgQPxDH5
</commit_message>
<xml_diff>
--- a/research/eu-shopovi-affiliate-hr.xlsx
+++ b/research/eu-shopovi-affiliate-hr.xlsx
@@ -7,14 +7,16 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Potvrđeni HR programi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EU shopovi – provjeriti HR" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ne dolazi u obzir" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EU bez HR verzije" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Potvrđeni HR programi" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EU shopovi – provjeriti HR" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ne dolazi u obzir" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Potvrđeni HR programi'!$A$1:$I$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'EU shopovi – provjeriti HR'!$A$1:$I$48</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Ne dolazi u obzir'!$A$1:$I$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'EU bez HR verzije'!$A$1:$H$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Potvrđeni HR programi'!$A$1:$I$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'EU shopovi – provjeriti HR'!$A$1:$I$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Ne dolazi u obzir'!$A$1:$I$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -448,6 +450,1585 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Shop</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Zemlja</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Kategorija</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Dokaz dostave u HR</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Mreža (program)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Provizija</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Cookie</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>3D Prima</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>3dprima.com</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>SE/DE</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Elektronika (3D printeri)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Hrvatska na popisu zemalja dostave</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler (3D Prima DE)</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>30 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>EcoFlow EU</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>eu.ecoflow.com</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>EU shop</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Elektronika (power stanice)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Croatia (EUR) u odabiru regije</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler (EcoFlow EU)</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>7 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>eufyMake (Anker)</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>eu.eufymake.com</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>EU shop</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Elektronika (UV printeri)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Croatia EUR u odabiru zemlje</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>30 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>GL.iNet</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>gl-inet.com</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>EU shop</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Elektronika (routeri)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Croatia EUR u europskoj regiji</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>45 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Marmitek</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>marmitek.com</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>NL</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Elektronika</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Hrvatska / Croatia (EUR) u odabiru zemlje</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler (Marmitek DE)</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>6%</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>30 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>eufy (SK shop)</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>sk.eufy.com</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>SK shop</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Elektronika</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Hrvatska na popisu dostave (3–7 dana)</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Awin, impact.com</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Amazon.de</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>amazon.de</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Sve kategorije</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Dostava u HR za dio artikala</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Amazon PartnerNet</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>po kategoriji</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>24 h</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Puma EU</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>eu.puma.com/hr/en</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Moda / sport</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Hrvatska na popisu dostave (engleski)</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>CJ</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Mytheresa</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>mytheresa.com</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Moda (luksuz)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Dostava u cijeli svijet</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Rakuten, CJ</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Tamaris</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>tamaris.com</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Moda / obuća</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Kroatien | HR (English)</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler (Tamaris DE)</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>7%</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>30 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>K-Swiss</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>kswiss.de</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Moda / tenisice</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Kroatien – Englisch – EUR</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler (K-Swiss DE)</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>6%</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>30 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Palladium</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>palladiumboots.de</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Moda / obuća</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Kroatien – Englisch – EUR</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler (Palladium DE)</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>30 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Gents</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>gents.de</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Moda (muška)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Kroatien na popisu zemalja</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>45 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Novoline Streetwear</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>shop.novoline.de</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Moda / streetwear</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Versand nach Kroatien (stranica dostave)</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>4%</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>30 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Woodstock Laundry</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>woodstocklaundry.eu</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Moda</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Croatia (EUR) u odabiru zemlje</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>30 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>AIMN</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>aimnsportswear.de</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>SE</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Moda / sportska odjeća</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Croatia na popisu zemalja</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>30 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Flattered</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>flattered.com</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>SE</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Moda / obuća</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Croatia EUR u odabiru zemlje</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>45 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Aubade</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>aubade.com</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Moda / donje rublje</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Croatia na popisu zemalja</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler (Aubade DE)</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>30 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Forte Forte</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>forte-forte.com</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Moda (premium)</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Croazia na popisu zemalja</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>30 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Gaelle Paris</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>gaelle.it</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Moda</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Croazia (EUR) u odabiru zemlje</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>12% novi</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>30 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Mood Fashion</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>moodfashion.com</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Moda</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Croazia EUR u odabiru zemlje</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>12%</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>45 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Quattro Stagioni</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>quattrostagionishop.com</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Moda</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Croazia na stranici dostave</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>30 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Loverlock</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>loverlock.it</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Moda / nakit</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Croazia (EUR) u odabiru zemlje</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>13%</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>30 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Toni Pons</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>tonipons.com</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Moda / espadrile</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Croacia (EUR) u odabiru zemlje</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler (Toni Pons IT)</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>9% novi</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>30 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Ulanka</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>ulanka.com</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Moda / obuća</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Croacia/HR na popisu zemalja</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler (Ulanka DE)</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>30 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Esdemarca</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>esdemarca.com</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Moda / obuća</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Croatia na popisu zemalja</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler (Esdemarca DE)</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>3%</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>30 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Naoko</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>naoko-store.pl</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Moda</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Chorwacja – dostava 36 zł</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>5,6%</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>30 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Sportstylestory</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>sportstylestory.com</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Moda / tenisice</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Chorwacja – 55 zł, 4–5 dana</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>6%</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>30 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Shoefresh</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>shoefresh.eu</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>NL</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Moda / njega obuće</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Croatia u odabiru zemlje dostave</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>10% novi</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>30 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>KIKO Milano</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>kikocosmetics.com</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Kozmetika</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Hrvatska: dostava 5,90 €, besplatno iznad 45 €</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>CJ, Awin</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Baro Cosmetics</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>barocosmetics.com</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Kozmetika</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Croazia EUR u odabiru zemlje</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>18%</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>45 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Eveline Cosmetics</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>eveline.pl</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Kozmetika</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Croatia (EUR) u odabiru zemlje</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>7%</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>30 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Judith Williams</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>judithwilliams.com</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Kozmetika</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Wir liefern … Kroatien (stranica dostave)</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>8% novi</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>30 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Feelgood Shop</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>feelgood-shop.com</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>NL/DE</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Kozmetika / zdravlje</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Kroatien na popisu zemalja dostave</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>30 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>More Nutrition</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>morenutrition.de</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Zdravlje / dodaci</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Kroatien na popisu zemalja</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>9% novi, 6% postojeći</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>30 dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Aurox Health</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>auroxhealth.com</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Zdravlje</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Croatia 4–5 dana, od 4,99 €</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Tradedoubler</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>4%</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>30 dana</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H37"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1247,7 +2828,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2985,7 +4566,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>